<commit_message>
fix start network monitor
</commit_message>
<xml_diff>
--- a/WpfUI/Resources/Templates/DotnetNetworking/Question/Environment.xlsx
+++ b/WpfUI/Resources/Templates/DotnetNetworking/Question/Environment.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnFall25\Code\Recorder_NetWorking\WpfUI\Resources\Templates\DotnetNetworking\Question\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15931C3F-DD1A-40E9-A5A3-870A185D66C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA833F9-4259-4D42-B8D0-B802DF0F7B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Config" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>Key</t>
   </si>
@@ -196,7 +196,19 @@
     <t>Given_Console_Host_Port</t>
   </si>
   <si>
-    <t>fptuxaes/aes-dotnet8-console</t>
+    <t>fptuxaes/aes-dotnet8-console:latest</t>
+  </si>
+  <si>
+    <t>Client</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>Meta\Given\Client</t>
+  </si>
+  <si>
+    <t>Meta\Given\Server</t>
   </si>
 </sst>
 </file>
@@ -814,17 +826,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="42.90625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.08984375" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.08984375" style="1"/>
+    <col min="1" max="1" width="30.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="42.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -832,7 +844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
@@ -840,7 +852,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>4</v>
       </c>
@@ -848,7 +860,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>6</v>
       </c>
@@ -856,7 +868,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>7</v>
       </c>
@@ -864,7 +876,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="18" t="s">
         <v>50</v>
       </c>
@@ -872,7 +884,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="20" t="s">
         <v>51</v>
       </c>
@@ -880,7 +892,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>8</v>
       </c>
@@ -888,31 +900,31 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>52</v>
       </c>
       <c r="B9" s="10"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>53</v>
       </c>
       <c r="B10" s="11"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>54</v>
       </c>
       <c r="B11" s="11"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>55</v>
       </c>
       <c r="B12" s="12"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>9</v>
       </c>
@@ -920,7 +932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>11</v>
       </c>
@@ -928,7 +940,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>13</v>
       </c>
@@ -936,7 +948,7 @@
         <v>1433</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>14</v>
       </c>
@@ -944,7 +956,7 @@
         <v>1434</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>15</v>
       </c>
@@ -952,7 +964,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>17</v>
       </c>
@@ -960,7 +972,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>19</v>
       </c>
@@ -968,7 +980,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>20</v>
       </c>
@@ -976,7 +988,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>22</v>
       </c>
@@ -984,17 +996,33 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="13"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
+      <c r="B24" s="13"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="15"/>
+      <c r="B25" s="15"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1007,14 +1035,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A83C95-3B80-4231-A2A3-554283AC2A02}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.6328125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="37.1796875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="37.21875" style="7" customWidth="1"/>
     <col min="3" max="3" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -1025,7 +1053,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>29</v>
       </c>
@@ -1036,7 +1064,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="22"/>
       <c r="B3" s="3" t="s">
         <v>32</v>
@@ -1045,7 +1073,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="22"/>
       <c r="B4" s="3" t="s">
         <v>34</v>
@@ -1054,7 +1082,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="22"/>
       <c r="B5" s="3" t="s">
         <v>36</v>
@@ -1063,7 +1091,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="22"/>
       <c r="B6" s="3" t="s">
         <v>38</v>
@@ -1072,7 +1100,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
         <v>40</v>
       </c>
@@ -1083,28 +1111,28 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="22"/>
       <c r="B8" s="3" t="s">
         <v>43</v>
       </c>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="22"/>
       <c r="B9" s="3" t="s">
         <v>44</v>
       </c>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="22"/>
       <c r="B10" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="24"/>
       <c r="B11" s="4" t="s">
         <v>46</v>

</xml_diff>